<commit_message>
update:Modul Pembahasan Hasil Asistensi
</commit_message>
<xml_diff>
--- a/avatar-apbd/excel/Laporan/Laporan Hasil Asistensi.xlsx
+++ b/avatar-apbd/excel/Laporan/Laporan Hasil Asistensi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\AVATARAPBD\avatar-apbd\excel\Laporan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{798AA984-30DC-4E01-B1BD-D26191358A17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3DE724F-886B-44A4-BE43-67967AA68C9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{0DC26B11-B0BE-44E9-BC95-A4B008C5514C}"/>
   </bookViews>
@@ -645,6 +645,7 @@
       <c r="G6" s="25"/>
       <c r="H6" s="25"/>
       <c r="I6" s="25"/>
+      <c r="J6" s="25"/>
     </row>
     <row r="7" spans="3:14" s="20" customFormat="1" x14ac:dyDescent="0.35">
       <c r="C7" s="1"/>
@@ -1243,7 +1244,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="D6:I6"/>
+    <mergeCell ref="D6:J6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>